<commit_message>
PSA/DPN patched version 20260630
</commit_message>
<xml_diff>
--- a/test26/xlsfiles/RAW-VARS.xlsx
+++ b/test26/xlsfiles/RAW-VARS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alfre\Github\kingair-Sys26-work\slcsos26\xlsfiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alfre\Github\kingair-Sys26-test\test26\xlsfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5A8AE7-FC0E-47F0-8DDB-9B930E05C694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719A808D-EFEE-424B-99EA-1D5E0ECDB4C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9912" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27240" yWindow="3435" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAS" sheetId="1" r:id="rId1"/>
@@ -450,43 +450,43 @@
     <t>DP2</t>
   </si>
   <si>
+    <t>PSB</t>
+  </si>
+  <si>
+    <t>PTB</t>
+  </si>
+  <si>
+    <t>BuckDewPoint</t>
+  </si>
+  <si>
+    <t>BuckPressure</t>
+  </si>
+  <si>
+    <t>BuckBoardTemp</t>
+  </si>
+  <si>
+    <t>BuckMirrorFlag</t>
+  </si>
+  <si>
+    <t>BuckDataFlag</t>
+  </si>
+  <si>
+    <t>TransducerOvenRTD</t>
+  </si>
+  <si>
+    <t>WaterBlockRTD</t>
+  </si>
+  <si>
+    <t>OAT1</t>
+  </si>
+  <si>
+    <t>PRES9000</t>
+  </si>
+  <si>
+    <t>DPN</t>
+  </si>
+  <si>
     <t>PSA</t>
-  </si>
-  <si>
-    <t>PSB</t>
-  </si>
-  <si>
-    <t>DPN</t>
-  </si>
-  <si>
-    <t>PTB</t>
-  </si>
-  <si>
-    <t>BuckDewPoint</t>
-  </si>
-  <si>
-    <t>BuckPressure</t>
-  </si>
-  <si>
-    <t>BuckBoardTemp</t>
-  </si>
-  <si>
-    <t>BuckMirrorFlag</t>
-  </si>
-  <si>
-    <t>BuckDataFlag</t>
-  </si>
-  <si>
-    <t>TransducerOvenRTD</t>
-  </si>
-  <si>
-    <t>WaterBlockRTD</t>
-  </si>
-  <si>
-    <t>OAT1</t>
-  </si>
-  <si>
-    <t>PRES9000</t>
   </si>
 </sst>
 </file>
@@ -849,23 +849,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="15" style="5" customWidth="1"/>
     <col min="5" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" customWidth="1"/>
-    <col min="11" max="11" width="9.109375" customWidth="1"/>
-    <col min="12" max="12" width="20.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" customWidth="1"/>
-    <col min="14" max="14" width="16.109375" customWidth="1"/>
-    <col min="15" max="15" width="12.33203125" customWidth="1"/>
-    <col min="17" max="17" width="12.33203125" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" customWidth="1"/>
+    <col min="12" max="12" width="20.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" customWidth="1"/>
+    <col min="14" max="14" width="16.140625" customWidth="1"/>
+    <col min="15" max="15" width="12.28515625" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>72</v>
       </c>
@@ -918,7 +918,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>73</v>
       </c>
@@ -971,7 +971,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>105</v>
       </c>
@@ -979,7 +979,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>5</v>
@@ -1007,7 +1007,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>2</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>139</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>140</v>
       </c>
@@ -1127,9 +1127,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="6" t="s">
@@ -1153,9 +1153,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="6" t="s">
@@ -1179,9 +1179,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="6" t="s">
@@ -1203,9 +1203,9 @@
       <c r="O10" s="4"/>
       <c r="Q10" s="4"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="6" t="s">
@@ -1227,9 +1227,9 @@
       <c r="O11" s="4"/>
       <c r="Q11" s="4"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="6" t="s">
@@ -1251,9 +1251,9 @@
       <c r="O12" s="4"/>
       <c r="Q12" s="4"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B13" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="6" t="s">
@@ -1275,9 +1275,9 @@
       <c r="O13" s="4"/>
       <c r="Q13" s="4"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="6" t="s">
@@ -1299,9 +1299,9 @@
       <c r="O14" s="4"/>
       <c r="Q14" s="4"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B15" s="7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="6" t="s">
@@ -1323,9 +1323,9 @@
       <c r="O15" s="4"/>
       <c r="Q15" s="4"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="6" t="s">
@@ -1347,9 +1347,9 @@
       <c r="O16" s="4"/>
       <c r="Q16" s="4"/>
     </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="6" t="s">
@@ -1371,9 +1371,9 @@
       <c r="O17" s="4"/>
       <c r="Q17" s="4"/>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="6" t="s">
@@ -1389,9 +1389,9 @@
       <c r="O18" s="4"/>
       <c r="Q18" s="4"/>
     </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B19" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="6" t="s">
@@ -1406,7 +1406,8 @@
       </c>
       <c r="Q19" s="4"/>
     </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B20" s="7"/>
       <c r="C20" s="1"/>
       <c r="D20" s="6" t="s">
         <v>22</v>
@@ -1420,7 +1421,7 @@
       </c>
       <c r="Q20" s="4"/>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B21" s="7"/>
       <c r="C21" s="1"/>
       <c r="D21" s="6" t="s">
@@ -1435,7 +1436,7 @@
       </c>
       <c r="Q21" s="4"/>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B22" s="7"/>
       <c r="C22" s="1"/>
       <c r="D22" s="6" t="s">
@@ -1450,7 +1451,7 @@
       </c>
       <c r="Q22" s="4"/>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B23" s="7"/>
       <c r="C23" s="1"/>
       <c r="D23" s="6" t="s">
@@ -1465,7 +1466,7 @@
       </c>
       <c r="Q23" s="4"/>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B24" s="7"/>
       <c r="C24" s="1"/>
       <c r="D24" s="6" t="s">
@@ -1479,7 +1480,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C25" s="1"/>
       <c r="D25" s="6" t="s">
         <v>27</v>
@@ -1492,7 +1493,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C26" s="1"/>
       <c r="D26" s="6" t="s">
         <v>28</v>
@@ -1505,80 +1506,80 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C27" s="1"/>
       <c r="J27" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C28" s="1"/>
       <c r="J28" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C29" s="1"/>
       <c r="J29" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C30" s="1"/>
       <c r="J30" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C31" s="1"/>
       <c r="J31" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C32" s="1"/>
       <c r="J32" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="33" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C33" s="1"/>
       <c r="J33" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C34" s="1"/>
       <c r="J34" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="35" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J35" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J36" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="37" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J37" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J38" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="39" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J39" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J40" s="2" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
Reference to dev* raw variables removed
</commit_message>
<xml_diff>
--- a/test26/xlsfiles/RAW-VARS.xlsx
+++ b/test26/xlsfiles/RAW-VARS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alfre\Github\kingair-Sys26-test\test26\xlsfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719A808D-EFEE-424B-99EA-1D5E0ECDB4C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5A8AE7-FC0E-47F0-8DDB-9B930E05C694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-27240" yWindow="3435" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -450,9 +450,15 @@
     <t>DP2</t>
   </si>
   <si>
+    <t>PSA</t>
+  </si>
+  <si>
     <t>PSB</t>
   </si>
   <si>
+    <t>DPN</t>
+  </si>
+  <si>
     <t>PTB</t>
   </si>
   <si>
@@ -481,12 +487,6 @@
   </si>
   <si>
     <t>PRES9000</t>
-  </si>
-  <si>
-    <t>DPN</t>
-  </si>
-  <si>
-    <t>PSA</t>
   </si>
 </sst>
 </file>
@@ -979,7 +979,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>5</v>
@@ -1129,7 +1129,7 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="6" t="s">
@@ -1155,7 +1155,7 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="6" t="s">
@@ -1181,7 +1181,7 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="6" t="s">
@@ -1205,7 +1205,7 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="6" t="s">
@@ -1229,7 +1229,7 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="6" t="s">
@@ -1253,7 +1253,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B13" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="6" t="s">
@@ -1277,7 +1277,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="6" t="s">
@@ -1301,7 +1301,7 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B15" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="6" t="s">
@@ -1325,7 +1325,7 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="6" t="s">
@@ -1349,7 +1349,7 @@
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="6" t="s">
@@ -1373,7 +1373,7 @@
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="6" t="s">
@@ -1391,7 +1391,7 @@
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B19" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="6" t="s">
@@ -1407,7 +1407,6 @@
       <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="7"/>
       <c r="C20" s="1"/>
       <c r="D20" s="6" t="s">
         <v>22</v>

</xml_diff>